<commit_message>
doc: slides with the results of the SVAR models
</commit_message>
<xml_diff>
--- a/doc/tablas coeficientes de sacrificio.xlsx
+++ b/doc/tablas coeficientes de sacrificio.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\OneDrive\Documents\github\VAR_estimation\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JGOR\Documents\github\VAR_estimation\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE844D52-BD98-44CF-BA21-989269DFE044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07A8116C-E2B8-4026-8F36-63AEE5988288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3020" yWindow="3020" windowWidth="19200" windowHeight="11180" xr2:uid="{24B9D59B-9ED4-437F-A292-A8E1645C3E3F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{24B9D59B-9ED4-437F-A292-A8E1645C3E3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Modelo</t>
   </si>
@@ -79,13 +78,44 @@
   </si>
   <si>
     <t>(-0.6677, 2.1664)</t>
+  </si>
+  <si>
+    <t>País</t>
+  </si>
+  <si>
+    <t>Coeficiente de sacrificio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estados Unidos  </t>
+  </si>
+  <si>
+    <t>Cecchetti and Robert (2001)</t>
+  </si>
+  <si>
+    <t>Zona Euro</t>
+  </si>
+  <si>
+    <t>Belke, Ansgar; Böing,
+Tobias (2007)</t>
+  </si>
+  <si>
+    <t>Italia</t>
+  </si>
+  <si>
+    <t>Francia</t>
+  </si>
+  <si>
+    <t>Países Bajos</t>
+  </si>
+  <si>
+    <t>España</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,7 +140,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -133,11 +163,92 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -146,6 +257,34 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -481,26 +620,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDFE5C68-1CC7-46CE-9C83-32166EFBE1FA}">
-  <dimension ref="B5:J10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B5:M19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6328125" customWidth="1"/>
-    <col min="10" max="10" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.625" customWidth="1"/>
+    <col min="10" max="10" width="25.375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.625" customWidth="1"/>
+    <col min="13" max="13" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:13" ht="15">
       <c r="C5" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:13" ht="15">
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
@@ -519,7 +660,7 @@
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:13" ht="15">
       <c r="B7" s="2">
         <v>1</v>
       </c>
@@ -545,7 +686,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:13">
       <c r="B8" s="2">
         <v>2</v>
       </c>
@@ -571,7 +712,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:13">
       <c r="B9" s="2">
         <v>3</v>
       </c>
@@ -597,7 +738,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:13" ht="14.25" customHeight="1">
       <c r="B10" s="2">
         <v>4</v>
       </c>
@@ -623,10 +764,77 @@
         <v>13</v>
       </c>
     </row>
+    <row r="11" spans="2:13" ht="45">
+      <c r="L11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13">
+      <c r="L12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="M12" s="8">
+        <v>1.3759999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" ht="28.5">
+      <c r="L13" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" s="10"/>
+    </row>
+    <row r="14" spans="2:13">
+      <c r="L14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="M14" s="12"/>
+    </row>
+    <row r="15" spans="2:13">
+      <c r="L15" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="M15" s="14"/>
+    </row>
+    <row r="16" spans="2:13">
+      <c r="L16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0.121</v>
+      </c>
+    </row>
+    <row r="17" spans="12:13">
+      <c r="L17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0.314</v>
+      </c>
+    </row>
+    <row r="18" spans="12:13">
+      <c r="L18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M18" s="2">
+        <v>1.323</v>
+      </c>
+    </row>
+    <row r="19" spans="12:13">
+      <c r="L19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M19" s="2">
+        <v>3.1070000000000002</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="H6:J6"/>
+    <mergeCell ref="L15:M15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>